<commit_message>
Actualización automática historial PIB
</commit_message>
<xml_diff>
--- a/monitoreo_pib.xlsx
+++ b/monitoreo_pib.xlsx
@@ -1214,7 +1214,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B40"/>
+  <dimension ref="A1:B41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1692,6 +1692,18 @@
         </is>
       </c>
       <c r="B40" t="inlineStr">
+        <is>
+          <t>Sin cambios</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>2026-09-20 17:14:40</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
         <is>
           <t>Sin cambios</t>
         </is>

</xml_diff>